<commit_message>
Add reviewed measurement faculty and separate research collaboration from mentorship
</commit_message>
<xml_diff>
--- a/site/exports/hit-shenzhen-ic.xlsx
+++ b/site/exports/hit-shenzhen-ic.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R462dcedfb73f4abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Re4004fa80baf45f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R4b0c3afb7b44455d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R120691efbcc24a4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R3a3ba9bcd6af4081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R42d2b2a480d74550"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Rf27eba33949d424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R60e46853139445e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R1258b71240ab40fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R2522062e50fe49ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T2_0" displayName="T2_0" ref="A1:G35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T3_0" displayName="T3_0" ref="A1:G35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T2_1" displayName="T2_1" ref="A1:Q234" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T3_1" displayName="T3_1" ref="A1:Q235" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="事件类型"/>
@@ -179,7 +179,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T2_2" displayName="T2_2" ref="A1:J34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T3_2" displayName="T3_2" ref="A1:J34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="导师姓名"/>
@@ -197,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T2_3" displayName="T2_3" ref="A1:J48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T3_3" displayName="T3_3" ref="A1:J48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="标题"/>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T2_4" displayName="T2_4" ref="A1:E142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T3_4" displayName="T3_4" ref="A1:E142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="来源ID"/>
@@ -1239,7 +1239,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdffb0872ff2140a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ab1adc560b4167"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8808,51 +8808,37 @@
     </x:row>
     <x:row r="196" ht="64" customHeight="1">
       <x:c r="A196" s="6" t="str">
-        <x:v>陈文君</x:v>
+        <x:v>张明宇</x:v>
       </x:c>
       <x:c r="B196" s="6" t="str">
-        <x:v>degree</x:v>
+        <x:v>research_assistant_collaborator</x:v>
       </x:c>
       <x:c r="C196" s="6" t="str">
-        <x:v>学士</x:v>
+        <x:v>研究助理阶段合作教授</x:v>
       </x:c>
       <x:c r="D196" s="6" t="str">
-        <x:v>大连理工大学</x:v>
+        <x:v>清华大学微纳米力学与多学科交叉创新研究中心</x:v>
       </x:c>
       <x:c r="E196" s="6" t="str">
-        <x:v>2009-09</x:v>
+        <x:v>2014-03</x:v>
       </x:c>
       <x:c r="F196" s="6" t="str">
-        <x:v>2013-07</x:v>
-      </x:c>
-      <x:c r="G196" s="6" t="str">
-        <x:v>Materials Processing and Control Engineering</x:v>
-      </x:c>
-      <x:c r="H196" s="6" t="str">
-        <x:v>中国</x:v>
-      </x:c>
-      <x:c r="I196" s="6" t="str">
-        <x:v>中国内地</x:v>
-      </x:c>
-      <x:c r="J196" s="6" t="str">
-        <x:v>亚洲</x:v>
-      </x:c>
-      <x:c r="K196" s="6" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="L196" s="13" t="b">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2014-08</x:v>
+      </x:c>
+      <x:c r="G196" s="6" t="str"/>
+      <x:c r="H196" s="6" t="str"/>
+      <x:c r="I196" s="6" t="str"/>
+      <x:c r="J196" s="6" t="str"/>
+      <x:c r="K196" s="6" t="str"/>
+      <x:c r="L196" s="6" t="str"/>
       <x:c r="M196" s="7" t="str"/>
       <x:c r="N196" s="6" t="str"/>
       <x:c r="O196" s="6" t="str">
-        <x:v>博士论文VITA xii页。</x:v>
-      </x:c>
-      <x:c r="P196" s="6" t="str">
-        <x:v>按来源所指院校所在地标准化，不代表国籍；授位与访问分开。</x:v>
-      </x:c>
+        <x:v>张莹莹；清华大学化学系教授、博士生导师，研究柔性可穿戴器件。；本人履历仅写合作教授，单列为研究合作，不声称学位导师。；非导师认定，不计师承；https://www.chem.tsinghua.edu.cn/info/1107/2644.htm</x:v>
+      </x:c>
+      <x:c r="P196" s="6" t="str"/>
       <x:c r="Q196" s="6" t="str">
-        <x:v>https://escholarship.org/content/qt3gm80490/qt3gm80490.pdf</x:v>
+        <x:v>https://homepage.hit.edu.cn/zhangmingyu</x:v>
       </x:c>
     </x:row>
     <x:row r="197" ht="64" customHeight="1">
@@ -8863,31 +8849,31 @@
         <x:v>degree</x:v>
       </x:c>
       <x:c r="C197" s="6" t="str">
-        <x:v>硕士</x:v>
+        <x:v>学士</x:v>
       </x:c>
       <x:c r="D197" s="6" t="str">
-        <x:v>加州大学默塞德分校</x:v>
+        <x:v>大连理工大学</x:v>
       </x:c>
       <x:c r="E197" s="6" t="str">
-        <x:v>2013-09</x:v>
+        <x:v>2009-09</x:v>
       </x:c>
       <x:c r="F197" s="6" t="str">
-        <x:v>2015-05</x:v>
+        <x:v>2013-07</x:v>
       </x:c>
       <x:c r="G197" s="6" t="str">
-        <x:v>Mechanical Engineering</x:v>
+        <x:v>Materials Processing and Control Engineering</x:v>
       </x:c>
       <x:c r="H197" s="6" t="str">
-        <x:v>美国</x:v>
+        <x:v>中国</x:v>
       </x:c>
       <x:c r="I197" s="6" t="str">
-        <x:v>美国</x:v>
+        <x:v>中国内地</x:v>
       </x:c>
       <x:c r="J197" s="6" t="str">
-        <x:v>北美洲</x:v>
+        <x:v>亚洲</x:v>
       </x:c>
       <x:c r="K197" s="6" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L197" s="13" t="b">
         <x:v>1</x:v>
@@ -8912,19 +8898,19 @@
         <x:v>degree</x:v>
       </x:c>
       <x:c r="C198" s="6" t="str">
-        <x:v>博士</x:v>
+        <x:v>硕士</x:v>
       </x:c>
       <x:c r="D198" s="6" t="str">
-        <x:v>加州大学圣地亚哥分校</x:v>
+        <x:v>加州大学默塞德分校</x:v>
       </x:c>
       <x:c r="E198" s="6" t="str">
-        <x:v>2015-09</x:v>
+        <x:v>2013-09</x:v>
       </x:c>
       <x:c r="F198" s="6" t="str">
-        <x:v>2019-12</x:v>
+        <x:v>2015-05</x:v>
       </x:c>
       <x:c r="G198" s="6" t="str">
-        <x:v>Materials Science and Engineering</x:v>
+        <x:v>Mechanical Engineering</x:v>
       </x:c>
       <x:c r="H198" s="6" t="str">
         <x:v>美国</x:v>
@@ -8944,7 +8930,7 @@
       <x:c r="M198" s="7" t="str"/>
       <x:c r="N198" s="6" t="str"/>
       <x:c r="O198" s="6" t="str">
-        <x:v>论文VITA给学习区间，封面与HIT官网确认2019博士，不另推精确授位日。</x:v>
+        <x:v>博士论文VITA xii页。</x:v>
       </x:c>
       <x:c r="P198" s="6" t="str">
         <x:v>按来源所指院校所在地标准化，不代表国籍；授位与访问分开。</x:v>
@@ -8958,30 +8944,48 @@
         <x:v>陈文君</x:v>
       </x:c>
       <x:c r="B199" s="6" t="str">
-        <x:v>employment</x:v>
+        <x:v>degree</x:v>
       </x:c>
       <x:c r="C199" s="6" t="str">
-        <x:v>Assistant Professor</x:v>
+        <x:v>博士</x:v>
       </x:c>
       <x:c r="D199" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）</x:v>
-      </x:c>
-      <x:c r="E199" s="6" t="str"/>
-      <x:c r="F199" s="6" t="str"/>
-      <x:c r="G199" s="6" t="str"/>
-      <x:c r="H199" s="6" t="str"/>
-      <x:c r="I199" s="6" t="str"/>
-      <x:c r="J199" s="6" t="str"/>
-      <x:c r="K199" s="6" t="str"/>
-      <x:c r="L199" s="6" t="str"/>
+        <x:v>加州大学圣地亚哥分校</x:v>
+      </x:c>
+      <x:c r="E199" s="6" t="str">
+        <x:v>2015-09</x:v>
+      </x:c>
+      <x:c r="F199" s="6" t="str">
+        <x:v>2019-12</x:v>
+      </x:c>
+      <x:c r="G199" s="6" t="str">
+        <x:v>Materials Science and Engineering</x:v>
+      </x:c>
+      <x:c r="H199" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I199" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J199" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K199" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L199" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="M199" s="7" t="str"/>
       <x:c r="N199" s="6" t="str"/>
       <x:c r="O199" s="6" t="str">
-        <x:v>英文个人简介现列Assistant Professor；学院副教授名录与其冲突，未擅自映射职级。</x:v>
-      </x:c>
-      <x:c r="P199" s="6" t="str"/>
+        <x:v>论文VITA给学习区间，封面与HIT官网确认2019博士，不另推精确授位日。</x:v>
+      </x:c>
+      <x:c r="P199" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位与访问分开。</x:v>
+      </x:c>
       <x:c r="Q199" s="6" t="str">
-        <x:v>https://homepage.hit.edu.cn/WenjunChen</x:v>
+        <x:v>https://escholarship.org/content/qt3gm80490/qt3gm80490.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="64" customHeight="1">
@@ -8992,10 +8996,10 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C200" s="6" t="str">
-        <x:v>副教授（名录类别）</x:v>
+        <x:v>Assistant Professor</x:v>
       </x:c>
       <x:c r="D200" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）集成电路学院</x:v>
+        <x:v>哈尔滨工业大学（深圳）</x:v>
       </x:c>
       <x:c r="E200" s="6" t="str"/>
       <x:c r="F200" s="6" t="str"/>
@@ -9008,11 +9012,11 @@
       <x:c r="M200" s="7" t="str"/>
       <x:c r="N200" s="6" t="str"/>
       <x:c r="O200" s="6" t="str">
-        <x:v>名录类别与个人英文Assistant Professor不一致，现职级待核。</x:v>
+        <x:v>英文个人简介现列Assistant Professor；学院副教授名录与其冲突，未擅自映射职级。</x:v>
       </x:c>
       <x:c r="P200" s="6" t="str"/>
       <x:c r="Q200" s="6" t="str">
-        <x:v>https://ic.hitsz.edu.cn/szll/qzjs/fjs.htm</x:v>
+        <x:v>https://homepage.hit.edu.cn/WenjunChen</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="64" customHeight="1">
@@ -9023,14 +9027,12 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C201" s="6" t="str">
-        <x:v>Graduate Researcher</x:v>
+        <x:v>副教授（名录类别）</x:v>
       </x:c>
       <x:c r="D201" s="6" t="str">
-        <x:v>加州大学圣地亚哥分校 Oscar Vazquez-Mena Lab</x:v>
-      </x:c>
-      <x:c r="E201" s="6" t="str">
-        <x:v>2015-09</x:v>
-      </x:c>
+        <x:v>哈尔滨工业大学（深圳）集成电路学院</x:v>
+      </x:c>
+      <x:c r="E201" s="6" t="str"/>
       <x:c r="F201" s="6" t="str"/>
       <x:c r="G201" s="6" t="str"/>
       <x:c r="H201" s="6" t="str"/>
@@ -9041,11 +9043,11 @@
       <x:c r="M201" s="7" t="str"/>
       <x:c r="N201" s="6" t="str"/>
       <x:c r="O201" s="6" t="str">
-        <x:v>论文VITA写2015-09至Present，Present指2019论文写作时，不表示当前仍在任；结束时间未披露。</x:v>
+        <x:v>名录类别与个人英文Assistant Professor不一致，现职级待核。</x:v>
       </x:c>
       <x:c r="P201" s="6" t="str"/>
       <x:c r="Q201" s="6" t="str">
-        <x:v>https://escholarship.org/content/qt3gm80490/qt3gm80490.pdf</x:v>
+        <x:v>https://ic.hitsz.edu.cn/szll/qzjs/fjs.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="64" customHeight="1">
@@ -9059,14 +9061,12 @@
         <x:v>Graduate Researcher</x:v>
       </x:c>
       <x:c r="D202" s="6" t="str">
-        <x:v>加州大学默塞德分校 Vincent C. Tung Lab</x:v>
+        <x:v>加州大学圣地亚哥分校 Oscar Vazquez-Mena Lab</x:v>
       </x:c>
       <x:c r="E202" s="6" t="str">
-        <x:v>2014-01</x:v>
-      </x:c>
-      <x:c r="F202" s="6" t="str">
-        <x:v>2015-05</x:v>
-      </x:c>
+        <x:v>2015-09</x:v>
+      </x:c>
+      <x:c r="F202" s="6" t="str"/>
       <x:c r="G202" s="6" t="str"/>
       <x:c r="H202" s="6" t="str"/>
       <x:c r="I202" s="6" t="str"/>
@@ -9076,7 +9076,7 @@
       <x:c r="M202" s="7" t="str"/>
       <x:c r="N202" s="6" t="str"/>
       <x:c r="O202" s="6" t="str">
-        <x:v>课题组研究身份，不据此推定硕士导师。</x:v>
+        <x:v>论文VITA写2015-09至Present，Present指2019论文写作时，不表示当前仍在任；结束时间未披露。</x:v>
       </x:c>
       <x:c r="P202" s="6" t="str"/>
       <x:c r="Q202" s="6" t="str">
@@ -9091,16 +9091,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C203" s="6" t="str">
-        <x:v>Teaching Assistant</x:v>
+        <x:v>Graduate Researcher</x:v>
       </x:c>
       <x:c r="D203" s="6" t="str">
-        <x:v>加州大学圣地亚哥分校</x:v>
+        <x:v>加州大学默塞德分校 Vincent C. Tung Lab</x:v>
       </x:c>
       <x:c r="E203" s="6" t="str">
-        <x:v>2017</x:v>
+        <x:v>2014-01</x:v>
       </x:c>
       <x:c r="F203" s="6" t="str">
-        <x:v>2019</x:v>
+        <x:v>2015-05</x:v>
       </x:c>
       <x:c r="G203" s="6" t="str"/>
       <x:c r="H203" s="6" t="str"/>
@@ -9111,7 +9111,7 @@
       <x:c r="M203" s="7" t="str"/>
       <x:c r="N203" s="6" t="str"/>
       <x:c r="O203" s="6" t="str">
-        <x:v>论文列Winter 2017/2018/2019，不表示连续全职任职。</x:v>
+        <x:v>课题组研究身份，不据此推定硕士导师。</x:v>
       </x:c>
       <x:c r="P203" s="6" t="str"/>
       <x:c r="Q203" s="6" t="str">
@@ -9129,13 +9129,13 @@
         <x:v>Teaching Assistant</x:v>
       </x:c>
       <x:c r="D204" s="6" t="str">
-        <x:v>加州大学默塞德分校</x:v>
+        <x:v>加州大学圣地亚哥分校</x:v>
       </x:c>
       <x:c r="E204" s="6" t="str">
-        <x:v>2013</x:v>
+        <x:v>2017</x:v>
       </x:c>
       <x:c r="F204" s="6" t="str">
-        <x:v>2015</x:v>
+        <x:v>2019</x:v>
       </x:c>
       <x:c r="G204" s="6" t="str"/>
       <x:c r="H204" s="6" t="str"/>
@@ -9146,7 +9146,7 @@
       <x:c r="M204" s="7" t="str"/>
       <x:c r="N204" s="6" t="str"/>
       <x:c r="O204" s="6" t="str">
-        <x:v>论文列2013/2014/2015。</x:v>
+        <x:v>论文列Winter 2017/2018/2019，不表示连续全职任职。</x:v>
       </x:c>
       <x:c r="P204" s="6" t="str"/>
       <x:c r="Q204" s="6" t="str">
@@ -9161,16 +9161,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C205" s="6" t="str">
-        <x:v>实习</x:v>
+        <x:v>Teaching Assistant</x:v>
       </x:c>
       <x:c r="D205" s="6" t="str">
-        <x:v>FAW Automobile Co., Ltd</x:v>
+        <x:v>加州大学默塞德分校</x:v>
       </x:c>
       <x:c r="E205" s="6" t="str">
-        <x:v>2012-07</x:v>
+        <x:v>2013</x:v>
       </x:c>
       <x:c r="F205" s="6" t="str">
-        <x:v>2012-09</x:v>
+        <x:v>2015</x:v>
       </x:c>
       <x:c r="G205" s="6" t="str"/>
       <x:c r="H205" s="6" t="str"/>
@@ -9180,7 +9180,9 @@
       <x:c r="L205" s="6" t="str"/>
       <x:c r="M205" s="7" t="str"/>
       <x:c r="N205" s="6" t="str"/>
-      <x:c r="O205" s="6" t="str"/>
+      <x:c r="O205" s="6" t="str">
+        <x:v>论文列2013/2014/2015。</x:v>
+      </x:c>
       <x:c r="P205" s="6" t="str"/>
       <x:c r="Q205" s="6" t="str">
         <x:v>https://escholarship.org/content/qt3gm80490/qt3gm80490.pdf</x:v>
@@ -9197,13 +9199,13 @@
         <x:v>实习</x:v>
       </x:c>
       <x:c r="D206" s="6" t="str">
-        <x:v>Chemical Fiber Group Co., Ltd</x:v>
+        <x:v>FAW Automobile Co., Ltd</x:v>
       </x:c>
       <x:c r="E206" s="6" t="str">
-        <x:v>2010-07</x:v>
+        <x:v>2012-07</x:v>
       </x:c>
       <x:c r="F206" s="6" t="str">
-        <x:v>2010-08</x:v>
+        <x:v>2012-09</x:v>
       </x:c>
       <x:c r="G206" s="6" t="str"/>
       <x:c r="H206" s="6" t="str"/>
@@ -9213,9 +9215,7 @@
       <x:c r="L206" s="6" t="str"/>
       <x:c r="M206" s="7" t="str"/>
       <x:c r="N206" s="6" t="str"/>
-      <x:c r="O206" s="6" t="str">
-        <x:v>机构原文未给更多身份，不自行扩写。</x:v>
-      </x:c>
+      <x:c r="O206" s="6" t="str"/>
       <x:c r="P206" s="6" t="str"/>
       <x:c r="Q206" s="6" t="str">
         <x:v>https://escholarship.org/content/qt3gm80490/qt3gm80490.pdf</x:v>
@@ -9223,49 +9223,37 @@
     </x:row>
     <x:row r="207" ht="64" customHeight="1">
       <x:c r="A207" s="6" t="str">
-        <x:v>祝温泊</x:v>
+        <x:v>陈文君</x:v>
       </x:c>
       <x:c r="B207" s="6" t="str">
-        <x:v>degree</x:v>
+        <x:v>employment</x:v>
       </x:c>
       <x:c r="C207" s="6" t="str">
-        <x:v>学士</x:v>
+        <x:v>实习</x:v>
       </x:c>
       <x:c r="D207" s="6" t="str">
-        <x:v>华中科技大学</x:v>
+        <x:v>Chemical Fiber Group Co., Ltd</x:v>
       </x:c>
       <x:c r="E207" s="6" t="str">
-        <x:v>2006-09</x:v>
+        <x:v>2010-07</x:v>
       </x:c>
       <x:c r="F207" s="6" t="str">
-        <x:v>2010-06</x:v>
-      </x:c>
-      <x:c r="G207" s="6" t="str">
-        <x:v>材料成型及控制工程</x:v>
-      </x:c>
-      <x:c r="H207" s="6" t="str">
-        <x:v>中国</x:v>
-      </x:c>
-      <x:c r="I207" s="6" t="str">
-        <x:v>中国内地</x:v>
-      </x:c>
-      <x:c r="J207" s="6" t="str">
-        <x:v>亚洲</x:v>
-      </x:c>
-      <x:c r="K207" s="6" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="L207" s="13" t="b">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2010-08</x:v>
+      </x:c>
+      <x:c r="G207" s="6" t="str"/>
+      <x:c r="H207" s="6" t="str"/>
+      <x:c r="I207" s="6" t="str"/>
+      <x:c r="J207" s="6" t="str"/>
+      <x:c r="K207" s="6" t="str"/>
+      <x:c r="L207" s="6" t="str"/>
       <x:c r="M207" s="7" t="str"/>
       <x:c r="N207" s="6" t="str"/>
-      <x:c r="O207" s="6" t="str"/>
-      <x:c r="P207" s="6" t="str">
-        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
-      </x:c>
+      <x:c r="O207" s="6" t="str">
+        <x:v>机构原文未给更多身份，不自行扩写。</x:v>
+      </x:c>
+      <x:c r="P207" s="6" t="str"/>
       <x:c r="Q207" s="6" t="str">
-        <x:v>https://homepage.hit.edu.cn/zhuwenbo</x:v>
+        <x:v>https://escholarship.org/content/qt3gm80490/qt3gm80490.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="64" customHeight="1">
@@ -9276,19 +9264,19 @@
         <x:v>degree</x:v>
       </x:c>
       <x:c r="C208" s="6" t="str">
-        <x:v>博士</x:v>
+        <x:v>学士</x:v>
       </x:c>
       <x:c r="D208" s="6" t="str">
         <x:v>华中科技大学</x:v>
       </x:c>
       <x:c r="E208" s="6" t="str">
-        <x:v>2010-09</x:v>
+        <x:v>2006-09</x:v>
       </x:c>
       <x:c r="F208" s="6" t="str">
-        <x:v>2017-03</x:v>
+        <x:v>2010-06</x:v>
       </x:c>
       <x:c r="G208" s="6" t="str">
-        <x:v>材料加工工程</x:v>
+        <x:v>材料成型及控制工程</x:v>
       </x:c>
       <x:c r="H208" s="6" t="str">
         <x:v>中国</x:v>
@@ -9302,12 +9290,12 @@
       <x:c r="K208" s="6" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="L208" s="6" t="str"/>
+      <x:c r="L208" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="M208" s="7" t="str"/>
       <x:c r="N208" s="6" t="str"/>
-      <x:c r="O208" s="6" t="str">
-        <x:v>官网列华中科技大学博士学习经历，与拉夫堡博士时间重叠；华科独立授位未获直接证实，degree_awarded保持null，不参与已确证博士授位统计，不推断联合培养或双学位。</x:v>
-      </x:c>
+      <x:c r="O208" s="6" t="str"/>
       <x:c r="P208" s="6" t="str">
         <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
       </x:c>
@@ -9326,35 +9314,35 @@
         <x:v>博士</x:v>
       </x:c>
       <x:c r="D209" s="6" t="str">
-        <x:v>Loughborough University</x:v>
+        <x:v>华中科技大学</x:v>
       </x:c>
       <x:c r="E209" s="6" t="str">
-        <x:v>2012-10</x:v>
+        <x:v>2010-09</x:v>
       </x:c>
       <x:c r="F209" s="6" t="str">
-        <x:v>2016-12</x:v>
+        <x:v>2017-03</x:v>
       </x:c>
       <x:c r="G209" s="6" t="str">
-        <x:v>Mechanical, Electrical and Manufacturing Engineering</x:v>
+        <x:v>材料加工工程</x:v>
       </x:c>
       <x:c r="H209" s="6" t="str">
-        <x:v>英国</x:v>
+        <x:v>中国</x:v>
       </x:c>
       <x:c r="I209" s="6" t="str">
-        <x:v>英国</x:v>
+        <x:v>中国内地</x:v>
       </x:c>
       <x:c r="J209" s="6" t="str">
-        <x:v>欧洲</x:v>
+        <x:v>亚洲</x:v>
       </x:c>
       <x:c r="K209" s="6" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="L209" s="13" t="b">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L209" s="6" t="str"/>
       <x:c r="M209" s="7" t="str"/>
       <x:c r="N209" s="6" t="str"/>
-      <x:c r="O209" s="6" t="str"/>
+      <x:c r="O209" s="6" t="str">
+        <x:v>官网列华中科技大学博士学习经历，与拉夫堡博士时间重叠；华科独立授位未获直接证实，degree_awarded保持null，不参与已确证博士授位统计，不推断联合培养或双学位。</x:v>
+      </x:c>
       <x:c r="P209" s="6" t="str">
         <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
       </x:c>
@@ -9367,30 +9355,44 @@
         <x:v>祝温泊</x:v>
       </x:c>
       <x:c r="B210" s="6" t="str">
-        <x:v>employment</x:v>
+        <x:v>degree</x:v>
       </x:c>
       <x:c r="C210" s="6" t="str">
-        <x:v>博士后</x:v>
+        <x:v>博士</x:v>
       </x:c>
       <x:c r="D210" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）</x:v>
+        <x:v>Loughborough University</x:v>
       </x:c>
       <x:c r="E210" s="6" t="str">
-        <x:v>2017-07</x:v>
+        <x:v>2012-10</x:v>
       </x:c>
       <x:c r="F210" s="6" t="str">
-        <x:v>2020-01</x:v>
-      </x:c>
-      <x:c r="G210" s="6" t="str"/>
-      <x:c r="H210" s="6" t="str"/>
-      <x:c r="I210" s="6" t="str"/>
-      <x:c r="J210" s="6" t="str"/>
-      <x:c r="K210" s="6" t="str"/>
-      <x:c r="L210" s="6" t="str"/>
+        <x:v>2016-12</x:v>
+      </x:c>
+      <x:c r="G210" s="6" t="str">
+        <x:v>Mechanical, Electrical and Manufacturing Engineering</x:v>
+      </x:c>
+      <x:c r="H210" s="6" t="str">
+        <x:v>英国</x:v>
+      </x:c>
+      <x:c r="I210" s="6" t="str">
+        <x:v>英国</x:v>
+      </x:c>
+      <x:c r="J210" s="6" t="str">
+        <x:v>欧洲</x:v>
+      </x:c>
+      <x:c r="K210" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L210" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="M210" s="7" t="str"/>
       <x:c r="N210" s="6" t="str"/>
       <x:c r="O210" s="6" t="str"/>
-      <x:c r="P210" s="6" t="str"/>
+      <x:c r="P210" s="6" t="str">
+        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
+      </x:c>
       <x:c r="Q210" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhuwenbo</x:v>
       </x:c>
@@ -9403,16 +9405,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C211" s="6" t="str">
-        <x:v>助理研究员</x:v>
+        <x:v>博士后</x:v>
       </x:c>
       <x:c r="D211" s="6" t="str">
         <x:v>哈尔滨工业大学（深圳）</x:v>
       </x:c>
       <x:c r="E211" s="6" t="str">
-        <x:v>2020-05</x:v>
+        <x:v>2017-07</x:v>
       </x:c>
       <x:c r="F211" s="6" t="str">
-        <x:v>2022-05</x:v>
+        <x:v>2020-01</x:v>
       </x:c>
       <x:c r="G211" s="6" t="str"/>
       <x:c r="H211" s="6" t="str"/>
@@ -9436,16 +9438,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C212" s="6" t="str">
-        <x:v>助理教授</x:v>
+        <x:v>助理研究员</x:v>
       </x:c>
       <x:c r="D212" s="6" t="str">
         <x:v>哈尔滨工业大学（深圳）</x:v>
       </x:c>
       <x:c r="E212" s="6" t="str">
+        <x:v>2020-05</x:v>
+      </x:c>
+      <x:c r="F212" s="6" t="str">
         <x:v>2022-05</x:v>
-      </x:c>
-      <x:c r="F212" s="6" t="str">
-        <x:v>2024-04</x:v>
       </x:c>
       <x:c r="G212" s="6" t="str"/>
       <x:c r="H212" s="6" t="str"/>
@@ -9469,16 +9471,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C213" s="6" t="str">
-        <x:v>副教授</x:v>
+        <x:v>助理教授</x:v>
       </x:c>
       <x:c r="D213" s="6" t="str">
         <x:v>哈尔滨工业大学（深圳）</x:v>
       </x:c>
       <x:c r="E213" s="6" t="str">
-        <x:v>2024-05</x:v>
+        <x:v>2022-05</x:v>
       </x:c>
       <x:c r="F213" s="6" t="str">
-        <x:v>2026-01</x:v>
+        <x:v>2024-04</x:v>
       </x:c>
       <x:c r="G213" s="6" t="str"/>
       <x:c r="H213" s="6" t="str"/>
@@ -9502,15 +9504,17 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C214" s="6" t="str">
-        <x:v>教授</x:v>
+        <x:v>副教授</x:v>
       </x:c>
       <x:c r="D214" s="6" t="str">
         <x:v>哈尔滨工业大学（深圳）</x:v>
       </x:c>
       <x:c r="E214" s="6" t="str">
-        <x:v>2026-02</x:v>
-      </x:c>
-      <x:c r="F214" s="6" t="str"/>
+        <x:v>2024-05</x:v>
+      </x:c>
+      <x:c r="F214" s="6" t="str">
+        <x:v>2026-01</x:v>
+      </x:c>
       <x:c r="G214" s="6" t="str"/>
       <x:c r="H214" s="6" t="str"/>
       <x:c r="I214" s="6" t="str"/>
@@ -9527,47 +9531,33 @@
     </x:row>
     <x:row r="215" ht="64" customHeight="1">
       <x:c r="A215" s="6" t="str">
-        <x:v>刘飞华</x:v>
+        <x:v>祝温泊</x:v>
       </x:c>
       <x:c r="B215" s="6" t="str">
-        <x:v>degree</x:v>
+        <x:v>employment</x:v>
       </x:c>
       <x:c r="C215" s="6" t="str">
-        <x:v>工学学士</x:v>
+        <x:v>教授</x:v>
       </x:c>
       <x:c r="D215" s="6" t="str">
-        <x:v>武汉理工大学</x:v>
+        <x:v>哈尔滨工业大学（深圳）</x:v>
       </x:c>
       <x:c r="E215" s="6" t="str">
-        <x:v>2008-09</x:v>
-      </x:c>
-      <x:c r="F215" s="6" t="str">
-        <x:v>2012-06</x:v>
-      </x:c>
+        <x:v>2026-02</x:v>
+      </x:c>
+      <x:c r="F215" s="6" t="str"/>
       <x:c r="G215" s="6" t="str"/>
-      <x:c r="H215" s="6" t="str">
-        <x:v>中国</x:v>
-      </x:c>
-      <x:c r="I215" s="6" t="str">
-        <x:v>中国内地</x:v>
-      </x:c>
-      <x:c r="J215" s="6" t="str">
-        <x:v>亚洲</x:v>
-      </x:c>
-      <x:c r="K215" s="6" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="L215" s="13" t="b">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H215" s="6" t="str"/>
+      <x:c r="I215" s="6" t="str"/>
+      <x:c r="J215" s="6" t="str"/>
+      <x:c r="K215" s="6" t="str"/>
+      <x:c r="L215" s="6" t="str"/>
       <x:c r="M215" s="7" t="str"/>
       <x:c r="N215" s="6" t="str"/>
       <x:c r="O215" s="6" t="str"/>
-      <x:c r="P215" s="6" t="str">
-        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
-      </x:c>
+      <x:c r="P215" s="6" t="str"/>
       <x:c r="Q215" s="6" t="str">
-        <x:v>https://homepage.hit.edu.cn/liufeihua</x:v>
+        <x:v>https://homepage.hit.edu.cn/zhuwenbo</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="64" customHeight="1">
@@ -9578,16 +9568,16 @@
         <x:v>degree</x:v>
       </x:c>
       <x:c r="C216" s="6" t="str">
-        <x:v>工学博士</x:v>
+        <x:v>工学学士</x:v>
       </x:c>
       <x:c r="D216" s="6" t="str">
         <x:v>武汉理工大学</x:v>
       </x:c>
       <x:c r="E216" s="6" t="str">
-        <x:v>2012-09</x:v>
+        <x:v>2008-09</x:v>
       </x:c>
       <x:c r="F216" s="6" t="str">
-        <x:v>2018-06</x:v>
+        <x:v>2012-06</x:v>
       </x:c>
       <x:c r="G216" s="6" t="str"/>
       <x:c r="H216" s="6" t="str">
@@ -9620,39 +9610,39 @@
         <x:v>刘飞华</x:v>
       </x:c>
       <x:c r="B217" s="6" t="str">
-        <x:v>joint_training</x:v>
-      </x:c>
-      <x:c r="C217" s="6" t="str"/>
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C217" s="6" t="str">
+        <x:v>工学博士</x:v>
+      </x:c>
       <x:c r="D217" s="6" t="str">
-        <x:v>The Pennsylvania State University</x:v>
+        <x:v>武汉理工大学</x:v>
       </x:c>
       <x:c r="E217" s="6" t="str">
-        <x:v>2014-09</x:v>
+        <x:v>2012-09</x:v>
       </x:c>
       <x:c r="F217" s="6" t="str">
-        <x:v>2017-06</x:v>
+        <x:v>2018-06</x:v>
       </x:c>
       <x:c r="G217" s="6" t="str"/>
       <x:c r="H217" s="6" t="str">
-        <x:v>美国</x:v>
+        <x:v>中国</x:v>
       </x:c>
       <x:c r="I217" s="6" t="str">
-        <x:v>美国</x:v>
+        <x:v>中国内地</x:v>
       </x:c>
       <x:c r="J217" s="6" t="str">
-        <x:v>北美洲</x:v>
+        <x:v>亚洲</x:v>
       </x:c>
       <x:c r="K217" s="6" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="L217" s="13" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M217" s="7" t="str"/>
       <x:c r="N217" s="6" t="str"/>
-      <x:c r="O217" s="6" t="str">
-        <x:v>官网明确联合培养博士；不认定为美国博士授位。</x:v>
-      </x:c>
+      <x:c r="O217" s="6" t="str"/>
       <x:c r="P217" s="6" t="str">
         <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
       </x:c>
@@ -9665,30 +9655,42 @@
         <x:v>刘飞华</x:v>
       </x:c>
       <x:c r="B218" s="6" t="str">
-        <x:v>employment</x:v>
-      </x:c>
-      <x:c r="C218" s="6" t="str">
-        <x:v>Research Associate</x:v>
-      </x:c>
+        <x:v>joint_training</x:v>
+      </x:c>
+      <x:c r="C218" s="6" t="str"/>
       <x:c r="D218" s="6" t="str">
-        <x:v>The Pennsylvania State University，材料科学与工程</x:v>
+        <x:v>The Pennsylvania State University</x:v>
       </x:c>
       <x:c r="E218" s="6" t="str">
-        <x:v>2016-09</x:v>
+        <x:v>2014-09</x:v>
       </x:c>
       <x:c r="F218" s="6" t="str">
         <x:v>2017-06</x:v>
       </x:c>
       <x:c r="G218" s="6" t="str"/>
-      <x:c r="H218" s="6" t="str"/>
-      <x:c r="I218" s="6" t="str"/>
-      <x:c r="J218" s="6" t="str"/>
-      <x:c r="K218" s="6" t="str"/>
-      <x:c r="L218" s="6" t="str"/>
+      <x:c r="H218" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I218" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J218" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K218" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L218" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="M218" s="7" t="str"/>
       <x:c r="N218" s="6" t="str"/>
-      <x:c r="O218" s="6" t="str"/>
-      <x:c r="P218" s="6" t="str"/>
+      <x:c r="O218" s="6" t="str">
+        <x:v>官网明确联合培养博士；不认定为美国博士授位。</x:v>
+      </x:c>
+      <x:c r="P218" s="6" t="str">
+        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
+      </x:c>
       <x:c r="Q218" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liufeihua</x:v>
       </x:c>
@@ -9701,16 +9703,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C219" s="6" t="str">
-        <x:v>研发总监/材料专家</x:v>
+        <x:v>Research Associate</x:v>
       </x:c>
       <x:c r="D219" s="6" t="str">
-        <x:v>深圳市信维通信股份有限公司中央研究院</x:v>
+        <x:v>The Pennsylvania State University，材料科学与工程</x:v>
       </x:c>
       <x:c r="E219" s="6" t="str">
-        <x:v>2018-07</x:v>
+        <x:v>2016-09</x:v>
       </x:c>
       <x:c r="F219" s="6" t="str">
-        <x:v>2021-06</x:v>
+        <x:v>2017-06</x:v>
       </x:c>
       <x:c r="G219" s="6" t="str"/>
       <x:c r="H219" s="6" t="str"/>
@@ -9734,16 +9736,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C220" s="6" t="str">
-        <x:v>助理研究员</x:v>
+        <x:v>研发总监/材料专家</x:v>
       </x:c>
       <x:c r="D220" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）材料科学与工程学院</x:v>
+        <x:v>深圳市信维通信股份有限公司中央研究院</x:v>
       </x:c>
       <x:c r="E220" s="6" t="str">
+        <x:v>2018-07</x:v>
+      </x:c>
+      <x:c r="F220" s="6" t="str">
         <x:v>2021-06</x:v>
-      </x:c>
-      <x:c r="F220" s="6" t="str">
-        <x:v>2023-12</x:v>
       </x:c>
       <x:c r="G220" s="6" t="str"/>
       <x:c r="H220" s="6" t="str"/>
@@ -9770,13 +9772,13 @@
         <x:v>助理研究员</x:v>
       </x:c>
       <x:c r="D221" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）集成电路学院</x:v>
+        <x:v>哈尔滨工业大学（深圳）材料科学与工程学院</x:v>
       </x:c>
       <x:c r="E221" s="6" t="str">
-        <x:v>2024-01</x:v>
+        <x:v>2021-06</x:v>
       </x:c>
       <x:c r="F221" s="6" t="str">
-        <x:v>2024-12</x:v>
+        <x:v>2023-12</x:v>
       </x:c>
       <x:c r="G221" s="6" t="str"/>
       <x:c r="H221" s="6" t="str"/>
@@ -9800,15 +9802,17 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C222" s="6" t="str">
-        <x:v>副研究员</x:v>
+        <x:v>助理研究员</x:v>
       </x:c>
       <x:c r="D222" s="6" t="str">
         <x:v>哈尔滨工业大学（深圳）集成电路学院</x:v>
       </x:c>
       <x:c r="E222" s="6" t="str">
+        <x:v>2024-01</x:v>
+      </x:c>
+      <x:c r="F222" s="6" t="str">
         <x:v>2024-12</x:v>
       </x:c>
-      <x:c r="F222" s="6" t="str"/>
       <x:c r="G222" s="6" t="str"/>
       <x:c r="H222" s="6" t="str"/>
       <x:c r="I222" s="6" t="str"/>
@@ -9825,47 +9829,33 @@
     </x:row>
     <x:row r="223" ht="64" customHeight="1">
       <x:c r="A223" s="6" t="str">
-        <x:v>李康</x:v>
+        <x:v>刘飞华</x:v>
       </x:c>
       <x:c r="B223" s="6" t="str">
-        <x:v>degree</x:v>
+        <x:v>employment</x:v>
       </x:c>
       <x:c r="C223" s="6" t="str">
-        <x:v>学士</x:v>
+        <x:v>副研究员</x:v>
       </x:c>
       <x:c r="D223" s="6" t="str">
-        <x:v>哈尔滨工业大学</x:v>
+        <x:v>哈尔滨工业大学（深圳）集成电路学院</x:v>
       </x:c>
       <x:c r="E223" s="6" t="str">
-        <x:v>2004-09</x:v>
-      </x:c>
-      <x:c r="F223" s="6" t="str">
-        <x:v>2008-07</x:v>
-      </x:c>
+        <x:v>2024-12</x:v>
+      </x:c>
+      <x:c r="F223" s="6" t="str"/>
       <x:c r="G223" s="6" t="str"/>
-      <x:c r="H223" s="6" t="str">
-        <x:v>中国</x:v>
-      </x:c>
-      <x:c r="I223" s="6" t="str">
-        <x:v>中国内地</x:v>
-      </x:c>
-      <x:c r="J223" s="6" t="str">
-        <x:v>亚洲</x:v>
-      </x:c>
-      <x:c r="K223" s="6" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="L223" s="13" t="b">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="H223" s="6" t="str"/>
+      <x:c r="I223" s="6" t="str"/>
+      <x:c r="J223" s="6" t="str"/>
+      <x:c r="K223" s="6" t="str"/>
+      <x:c r="L223" s="6" t="str"/>
       <x:c r="M223" s="7" t="str"/>
       <x:c r="N223" s="6" t="str"/>
       <x:c r="O223" s="6" t="str"/>
-      <x:c r="P223" s="6" t="str">
-        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
-      </x:c>
+      <x:c r="P223" s="6" t="str"/>
       <x:c r="Q223" s="6" t="str">
-        <x:v>https://homepage.hit.edu.cn/likang</x:v>
+        <x:v>https://homepage.hit.edu.cn/liufeihua</x:v>
       </x:c>
     </x:row>
     <x:row r="224" ht="64" customHeight="1">
@@ -9876,16 +9866,16 @@
         <x:v>degree</x:v>
       </x:c>
       <x:c r="C224" s="6" t="str">
-        <x:v>博士</x:v>
+        <x:v>学士</x:v>
       </x:c>
       <x:c r="D224" s="6" t="str">
-        <x:v>中国科学院物理研究所</x:v>
+        <x:v>哈尔滨工业大学</x:v>
       </x:c>
       <x:c r="E224" s="6" t="str">
-        <x:v>2008-09</x:v>
+        <x:v>2004-09</x:v>
       </x:c>
       <x:c r="F224" s="6" t="str">
-        <x:v>2015-01</x:v>
+        <x:v>2008-07</x:v>
       </x:c>
       <x:c r="G224" s="6" t="str"/>
       <x:c r="H224" s="6" t="str">
@@ -9898,16 +9888,14 @@
         <x:v>亚洲</x:v>
       </x:c>
       <x:c r="K224" s="6" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L224" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="M224" s="7" t="str"/>
       <x:c r="N224" s="6" t="str"/>
-      <x:c r="O224" s="6" t="str">
-        <x:v>官网以中科院物理研究所列学位经历；未将授位机构自动改成中国科学院大学。</x:v>
-      </x:c>
+      <x:c r="O224" s="6" t="str"/>
       <x:c r="P224" s="6" t="str">
         <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
       </x:c>
@@ -9920,30 +9908,44 @@
         <x:v>李康</x:v>
       </x:c>
       <x:c r="B225" s="6" t="str">
-        <x:v>employment</x:v>
+        <x:v>degree</x:v>
       </x:c>
       <x:c r="C225" s="6" t="str">
-        <x:v>博士后</x:v>
+        <x:v>博士</x:v>
       </x:c>
       <x:c r="D225" s="6" t="str">
-        <x:v>清华大学物理系</x:v>
+        <x:v>中国科学院物理研究所</x:v>
       </x:c>
       <x:c r="E225" s="6" t="str">
-        <x:v>2015-04</x:v>
+        <x:v>2008-09</x:v>
       </x:c>
       <x:c r="F225" s="6" t="str">
-        <x:v>2017-04</x:v>
+        <x:v>2015-01</x:v>
       </x:c>
       <x:c r="G225" s="6" t="str"/>
-      <x:c r="H225" s="6" t="str"/>
-      <x:c r="I225" s="6" t="str"/>
-      <x:c r="J225" s="6" t="str"/>
-      <x:c r="K225" s="6" t="str"/>
-      <x:c r="L225" s="6" t="str"/>
+      <x:c r="H225" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I225" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J225" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K225" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L225" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="M225" s="7" t="str"/>
       <x:c r="N225" s="6" t="str"/>
-      <x:c r="O225" s="6" t="str"/>
-      <x:c r="P225" s="6" t="str"/>
+      <x:c r="O225" s="6" t="str">
+        <x:v>官网以中科院物理研究所列学位经历；未将授位机构自动改成中国科学院大学。</x:v>
+      </x:c>
+      <x:c r="P225" s="6" t="str">
+        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
+      </x:c>
       <x:c r="Q225" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/likang</x:v>
       </x:c>
@@ -9956,16 +9958,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C226" s="6" t="str">
-        <x:v>技术总监</x:v>
+        <x:v>博士后</x:v>
       </x:c>
       <x:c r="D226" s="6" t="str">
-        <x:v>苏州来福易材料科技有限公司</x:v>
+        <x:v>清华大学物理系</x:v>
       </x:c>
       <x:c r="E226" s="6" t="str">
-        <x:v>2017-05</x:v>
+        <x:v>2015-04</x:v>
       </x:c>
       <x:c r="F226" s="6" t="str">
-        <x:v>2019-04</x:v>
+        <x:v>2017-04</x:v>
       </x:c>
       <x:c r="G226" s="6" t="str"/>
       <x:c r="H226" s="6" t="str"/>
@@ -9989,13 +9991,17 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C227" s="6" t="str">
-        <x:v>助理研究员</x:v>
+        <x:v>技术总监</x:v>
       </x:c>
       <x:c r="D227" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）柔性印刷电子技术研究中心</x:v>
-      </x:c>
-      <x:c r="E227" s="6" t="str"/>
-      <x:c r="F227" s="6" t="str"/>
+        <x:v>苏州来福易材料科技有限公司</x:v>
+      </x:c>
+      <x:c r="E227" s="6" t="str">
+        <x:v>2017-05</x:v>
+      </x:c>
+      <x:c r="F227" s="6" t="str">
+        <x:v>2019-04</x:v>
+      </x:c>
       <x:c r="G227" s="6" t="str"/>
       <x:c r="H227" s="6" t="str"/>
       <x:c r="I227" s="6" t="str"/>
@@ -10004,9 +10010,7 @@
       <x:c r="L227" s="6" t="str"/>
       <x:c r="M227" s="7" t="str"/>
       <x:c r="N227" s="6" t="str"/>
-      <x:c r="O227" s="6" t="str">
-        <x:v>主页个人简介列此职称；名录列研究员类别，不将类别强制改成正研究员。</x:v>
-      </x:c>
+      <x:c r="O227" s="6" t="str"/>
       <x:c r="P227" s="6" t="str"/>
       <x:c r="Q227" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/likang</x:v>
@@ -10014,49 +10018,33 @@
     </x:row>
     <x:row r="228" ht="64" customHeight="1">
       <x:c r="A228" s="6" t="str">
-        <x:v>冯欢欢</x:v>
+        <x:v>李康</x:v>
       </x:c>
       <x:c r="B228" s="6" t="str">
-        <x:v>degree</x:v>
+        <x:v>employment</x:v>
       </x:c>
       <x:c r="C228" s="6" t="str">
-        <x:v>学士</x:v>
+        <x:v>助理研究员</x:v>
       </x:c>
       <x:c r="D228" s="6" t="str">
-        <x:v>北京师范大学</x:v>
-      </x:c>
-      <x:c r="E228" s="6" t="str">
-        <x:v>2002-09</x:v>
-      </x:c>
-      <x:c r="F228" s="6" t="str">
-        <x:v>2006-07</x:v>
-      </x:c>
-      <x:c r="G228" s="6" t="str">
-        <x:v>化学学院（院系名）</x:v>
-      </x:c>
-      <x:c r="H228" s="6" t="str">
-        <x:v>中国</x:v>
-      </x:c>
-      <x:c r="I228" s="6" t="str">
-        <x:v>中国内地</x:v>
-      </x:c>
-      <x:c r="J228" s="6" t="str">
-        <x:v>亚洲</x:v>
-      </x:c>
-      <x:c r="K228" s="6" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="L228" s="13" t="b">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>哈尔滨工业大学（深圳）柔性印刷电子技术研究中心</x:v>
+      </x:c>
+      <x:c r="E228" s="6" t="str"/>
+      <x:c r="F228" s="6" t="str"/>
+      <x:c r="G228" s="6" t="str"/>
+      <x:c r="H228" s="6" t="str"/>
+      <x:c r="I228" s="6" t="str"/>
+      <x:c r="J228" s="6" t="str"/>
+      <x:c r="K228" s="6" t="str"/>
+      <x:c r="L228" s="6" t="str"/>
       <x:c r="M228" s="7" t="str"/>
       <x:c r="N228" s="6" t="str"/>
-      <x:c r="O228" s="6" t="str"/>
-      <x:c r="P228" s="6" t="str">
-        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
-      </x:c>
+      <x:c r="O228" s="6" t="str">
+        <x:v>主页个人简介列此职称；名录列研究员类别，不将类别强制改成正研究员。</x:v>
+      </x:c>
+      <x:c r="P228" s="6" t="str"/>
       <x:c r="Q228" s="6" t="str">
-        <x:v>https://homepage.hit.edu.cn/fenghuanhuan</x:v>
+        <x:v>https://homepage.hit.edu.cn/likang</x:v>
       </x:c>
     </x:row>
     <x:row r="229" ht="64" customHeight="1">
@@ -10067,19 +10055,19 @@
         <x:v>degree</x:v>
       </x:c>
       <x:c r="C229" s="6" t="str">
-        <x:v>硕士</x:v>
+        <x:v>学士</x:v>
       </x:c>
       <x:c r="D229" s="6" t="str">
         <x:v>北京师范大学</x:v>
       </x:c>
       <x:c r="E229" s="6" t="str">
-        <x:v>2006-09</x:v>
+        <x:v>2002-09</x:v>
       </x:c>
       <x:c r="F229" s="6" t="str">
-        <x:v>2009-07</x:v>
+        <x:v>2006-07</x:v>
       </x:c>
       <x:c r="G229" s="6" t="str">
-        <x:v>高分子物理化学研究组（研究组名）</x:v>
+        <x:v>化学学院（院系名）</x:v>
       </x:c>
       <x:c r="H229" s="6" t="str">
         <x:v>中国</x:v>
@@ -10114,42 +10102,38 @@
         <x:v>degree</x:v>
       </x:c>
       <x:c r="C230" s="6" t="str">
-        <x:v>博士</x:v>
+        <x:v>硕士</x:v>
       </x:c>
       <x:c r="D230" s="6" t="str">
-        <x:v>Wageningen University</x:v>
+        <x:v>北京师范大学</x:v>
       </x:c>
       <x:c r="E230" s="6" t="str">
-        <x:v>2009-09</x:v>
+        <x:v>2006-09</x:v>
       </x:c>
       <x:c r="F230" s="6" t="str">
-        <x:v>2013-09</x:v>
+        <x:v>2009-07</x:v>
       </x:c>
       <x:c r="G230" s="6" t="str">
-        <x:v>Physical Chemistry and Soft Matter（机构名）</x:v>
+        <x:v>高分子物理化学研究组（研究组名）</x:v>
       </x:c>
       <x:c r="H230" s="6" t="str">
-        <x:v>荷兰</x:v>
+        <x:v>中国</x:v>
       </x:c>
       <x:c r="I230" s="6" t="str">
-        <x:v>荷兰</x:v>
+        <x:v>中国内地</x:v>
       </x:c>
       <x:c r="J230" s="6" t="str">
-        <x:v>欧洲</x:v>
+        <x:v>亚洲</x:v>
       </x:c>
       <x:c r="K230" s="6" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="L230" s="13" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M230" s="7" t="d">
-        <x:v>2013-12-09T00:00:00.000Z</x:v>
-      </x:c>
+      <x:c r="M230" s="7" t="str"/>
       <x:c r="N230" s="6" t="str"/>
-      <x:c r="O230" s="6" t="str">
-        <x:v>HIT履历结束日期2013-09；WUR学位库明确授位2013-12-09，另存degree_awarded_date，不用履历结束日期代替授位日。</x:v>
-      </x:c>
+      <x:c r="O230" s="6" t="str"/>
       <x:c r="P230" s="6" t="str">
         <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
       </x:c>
@@ -10162,30 +10146,48 @@
         <x:v>冯欢欢</x:v>
       </x:c>
       <x:c r="B231" s="6" t="str">
-        <x:v>employment</x:v>
+        <x:v>degree</x:v>
       </x:c>
       <x:c r="C231" s="6" t="str">
-        <x:v>博士后</x:v>
+        <x:v>博士</x:v>
       </x:c>
       <x:c r="D231" s="6" t="str">
-        <x:v>Wageningen University，Physical Chemistry and Soft Matter</x:v>
+        <x:v>Wageningen University</x:v>
       </x:c>
       <x:c r="E231" s="6" t="str">
+        <x:v>2009-09</x:v>
+      </x:c>
+      <x:c r="F231" s="6" t="str">
         <x:v>2013-09</x:v>
       </x:c>
-      <x:c r="F231" s="6" t="str">
-        <x:v>2016-09</x:v>
-      </x:c>
-      <x:c r="G231" s="6" t="str"/>
-      <x:c r="H231" s="6" t="str"/>
-      <x:c r="I231" s="6" t="str"/>
-      <x:c r="J231" s="6" t="str"/>
-      <x:c r="K231" s="6" t="str"/>
-      <x:c r="L231" s="6" t="str"/>
-      <x:c r="M231" s="7" t="str"/>
+      <x:c r="G231" s="6" t="str">
+        <x:v>Physical Chemistry and Soft Matter（机构名）</x:v>
+      </x:c>
+      <x:c r="H231" s="6" t="str">
+        <x:v>荷兰</x:v>
+      </x:c>
+      <x:c r="I231" s="6" t="str">
+        <x:v>荷兰</x:v>
+      </x:c>
+      <x:c r="J231" s="6" t="str">
+        <x:v>欧洲</x:v>
+      </x:c>
+      <x:c r="K231" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L231" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M231" s="7" t="d">
+        <x:v>2013-12-09T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="N231" s="6" t="str"/>
-      <x:c r="O231" s="6" t="str"/>
-      <x:c r="P231" s="6" t="str"/>
+      <x:c r="O231" s="6" t="str">
+        <x:v>HIT履历结束日期2013-09；WUR学位库明确授位2013-12-09，另存degree_awarded_date，不用履历结束日期代替授位日。</x:v>
+      </x:c>
+      <x:c r="P231" s="6" t="str">
+        <x:v>按院校所在地标准化，不代表国籍；非授位访问与联合培养单列。</x:v>
+      </x:c>
       <x:c r="Q231" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/fenghuanhuan</x:v>
       </x:c>
@@ -10198,16 +10200,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C232" s="6" t="str">
-        <x:v>助理教授</x:v>
+        <x:v>博士后</x:v>
       </x:c>
       <x:c r="D232" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）材料科学与工程学院</x:v>
+        <x:v>Wageningen University，Physical Chemistry and Soft Matter</x:v>
       </x:c>
       <x:c r="E232" s="6" t="str">
+        <x:v>2013-09</x:v>
+      </x:c>
+      <x:c r="F232" s="6" t="str">
         <x:v>2016-09</x:v>
-      </x:c>
-      <x:c r="F232" s="6" t="str">
-        <x:v>2022-09</x:v>
       </x:c>
       <x:c r="G232" s="6" t="str"/>
       <x:c r="H232" s="6" t="str"/>
@@ -10231,16 +10233,16 @@
         <x:v>employment</x:v>
       </x:c>
       <x:c r="C233" s="6" t="str">
-        <x:v>副研究员</x:v>
+        <x:v>助理教授</x:v>
       </x:c>
       <x:c r="D233" s="6" t="str">
         <x:v>哈尔滨工业大学（深圳）材料科学与工程学院</x:v>
       </x:c>
       <x:c r="E233" s="6" t="str">
+        <x:v>2016-09</x:v>
+      </x:c>
+      <x:c r="F233" s="6" t="str">
         <x:v>2022-09</x:v>
-      </x:c>
-      <x:c r="F233" s="6" t="str">
-        <x:v>2024-06</x:v>
       </x:c>
       <x:c r="G233" s="6" t="str"/>
       <x:c r="H233" s="6" t="str"/>
@@ -10267,12 +10269,14 @@
         <x:v>副研究员</x:v>
       </x:c>
       <x:c r="D234" s="6" t="str">
-        <x:v>哈尔滨工业大学（深圳）集成电路学院</x:v>
+        <x:v>哈尔滨工业大学（深圳）材料科学与工程学院</x:v>
       </x:c>
       <x:c r="E234" s="6" t="str">
+        <x:v>2022-09</x:v>
+      </x:c>
+      <x:c r="F234" s="6" t="str">
         <x:v>2024-06</x:v>
       </x:c>
-      <x:c r="F234" s="6" t="str"/>
       <x:c r="G234" s="6" t="str"/>
       <x:c r="H234" s="6" t="str"/>
       <x:c r="I234" s="6" t="str"/>
@@ -10287,10 +10291,41 @@
         <x:v>https://homepage.hit.edu.cn/fenghuanhuan</x:v>
       </x:c>
     </x:row>
+    <x:row r="235" ht="64" customHeight="1">
+      <x:c r="A235" s="6" t="str">
+        <x:v>冯欢欢</x:v>
+      </x:c>
+      <x:c r="B235" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C235" s="6" t="str">
+        <x:v>副研究员</x:v>
+      </x:c>
+      <x:c r="D235" s="6" t="str">
+        <x:v>哈尔滨工业大学（深圳）集成电路学院</x:v>
+      </x:c>
+      <x:c r="E235" s="6" t="str">
+        <x:v>2024-06</x:v>
+      </x:c>
+      <x:c r="F235" s="6" t="str"/>
+      <x:c r="G235" s="6" t="str"/>
+      <x:c r="H235" s="6" t="str"/>
+      <x:c r="I235" s="6" t="str"/>
+      <x:c r="J235" s="6" t="str"/>
+      <x:c r="K235" s="6" t="str"/>
+      <x:c r="L235" s="6" t="str"/>
+      <x:c r="M235" s="7" t="str"/>
+      <x:c r="N235" s="6" t="str"/>
+      <x:c r="O235" s="6" t="str"/>
+      <x:c r="P235" s="6" t="str"/>
+      <x:c r="Q235" s="6" t="str">
+        <x:v>https://homepage.hit.edu.cn/fenghuanhuan</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cf10e59ff494588"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc759782815714087"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11382,7 +11417,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ca7b80ca99d4082"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b76877c4c90494e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12848,7 +12883,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recdb81b588484319"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re947935b5fa74edb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15281,7 +15316,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea61e84ad34b47ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0d7c7a6f8ba4e87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>